<commit_message>
clean up remaining renamed and converted files across project
</commit_message>
<xml_diff>
--- a/Research Assets/Engagement Metrics/Engagement ContentAnalysis Merged.xlsx
+++ b/Research Assets/Engagement Metrics/Engagement ContentAnalysis Merged.xlsx
@@ -20551,7 +20551,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Banky Wellington</t>
+          <t>Banky Wellington | Ebuka Obi-Uchendu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20560,7 +20560,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -20588,7 +20588,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Banky Wellington</t>
+          <t>Banky Wellington | Ebuka Obi-Uchendu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20597,7 +20597,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -20625,7 +20625,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Banky Wellington</t>
+          <t>Banky Wellington | Ebuka Obi-Uchendu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -20634,7 +20634,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -20662,7 +20662,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Banky Wellington</t>
+          <t>Banky Wellington | Ebuka Obi-Uchendu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -20671,7 +20671,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -20699,7 +20699,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Banky Wellington</t>
+          <t>Banky Wellington | Ebuka Obi-Uchendu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -20708,7 +20708,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>

</xml_diff>